<commit_message>
update fce a 2 lekce faktory
</commit_message>
<xml_diff>
--- a/domaciUkoly/odevzdání.xlsx
+++ b/domaciUkoly/odevzdání.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucie Hošková\Desktop\introR_CUNI\domaciUkoly\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1B7CEF7-C304-4575-9175-0ECC80025DAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A364C2D-9C58-49F5-8466-A9D97B0DED8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01'!$A$1:$B$17</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -25,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Odevzdáno</t>
   </si>
@@ -37,6 +40,39 @@
   </si>
   <si>
     <t>Jméno</t>
+  </si>
+  <si>
+    <t>Jana Neubert</t>
+  </si>
+  <si>
+    <t>Nikola Ternerová</t>
+  </si>
+  <si>
+    <t>Anna Svěráková</t>
+  </si>
+  <si>
+    <t>Klára Tučková</t>
+  </si>
+  <si>
+    <t>Lenka Nosková</t>
+  </si>
+  <si>
+    <t>Valerie Grobarová</t>
+  </si>
+  <si>
+    <t>Andrea Hudousková</t>
+  </si>
+  <si>
+    <t>Markéta Pokorná</t>
+  </si>
+  <si>
+    <t>Fillip Weisz</t>
+  </si>
+  <si>
+    <t>Natálie Hříbková</t>
+  </si>
+  <si>
+    <t>Lenka Doubravská</t>
   </si>
 </sst>
 </file>
@@ -381,7 +417,7 @@
   <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.90625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -395,7 +431,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="B2" s="1" t="b">
         <v>1</v>
@@ -403,65 +439,98 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B3" s="1" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
       <c r="B4" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
       <c r="B5" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
       <c r="B6" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
       <c r="B7" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
       <c r="B8" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
       <c r="B9" s="1" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
       <c r="B10" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
       <c r="B11" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>1</v>
+      </c>
       <c r="B12" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
       <c r="B13" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>2</v>
+      </c>
       <c r="B14" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
@@ -480,6 +549,11 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B17" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B17">
+      <sortCondition ref="A1:A17"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
1 uprava info 2 uprava faktory 3 hotovo
</commit_message>
<xml_diff>
--- a/domaciUkoly/odevzdání.xlsx
+++ b/domaciUkoly/odevzdání.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hoskovalucie2\introR_CUNI\domaciUkoly\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucie Hošková\Desktop\introR_CUNI\domaciUkoly\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02234B61-B262-41C1-B0A9-6724FD71D954}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0CD50D8-A87A-4846-B2B5-7C13BF881C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="odevzdáno" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Sam Herczeg</t>
   </si>
@@ -72,9 +72,6 @@
     <t>Lenka Doubravská</t>
   </si>
   <si>
-    <t>Magdalena H. Medová</t>
-  </si>
-  <si>
     <t>Eva Kamenná</t>
   </si>
   <si>
@@ -82,6 +79,12 @@
   </si>
   <si>
     <t>1. hodina</t>
+  </si>
+  <si>
+    <t>2. hodina</t>
+  </si>
+  <si>
+    <t>Magdalena H. Megová</t>
   </si>
 </sst>
 </file>
@@ -423,146 +426,197 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.86328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>2</v>
       </c>
       <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C2" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C3" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C4" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C5" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C6" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C7" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C8" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>7</v>
       </c>
       <c r="B9" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C9" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B10" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C10" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="C11" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>12</v>
       </c>
       <c r="B12" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C12" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>4</v>
       </c>
       <c r="B13" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C13" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>0</v>
       </c>
       <c r="B14" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C14" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>8</v>
       </c>
       <c r="B15" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C15" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>1</v>
       </c>
       <c r="B16" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C16" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="C17" s="1" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
3 beta read 3 dodani materialu
</commit_message>
<xml_diff>
--- a/domaciUkoly/odevzdání.xlsx
+++ b/domaciUkoly/odevzdání.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucie Hošková\Desktop\introR_CUNI\domaciUkoly\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0CD50D8-A87A-4846-B2B5-7C13BF881C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95E0C616-2253-453B-81E9-96A9949F4B81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -474,7 +474,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
4 uprava presun do tipy
</commit_message>
<xml_diff>
--- a/domaciUkoly/odevzdání.xlsx
+++ b/domaciUkoly/odevzdání.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucie Hošková\Desktop\introR_CUNI\domaciUkoly\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95E0C616-2253-453B-81E9-96A9949F4B81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B9D549D-D7D4-43A6-9E08-0776603196B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="odevzdáno" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Sam Herczeg</t>
   </si>
@@ -85,6 +85,9 @@
   </si>
   <si>
     <t>Magdalena H. Megová</t>
+  </si>
+  <si>
+    <t>3. hodina</t>
   </si>
 </sst>
 </file>
@@ -426,14 +429,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.86328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -443,8 +446,11 @@
       <c r="C1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -454,8 +460,11 @@
       <c r="C2" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D2" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -465,8 +474,11 @@
       <c r="C3" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D3" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -476,8 +488,11 @@
       <c r="C4" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D4" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -487,8 +502,11 @@
       <c r="C5" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D5" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -498,8 +516,11 @@
       <c r="C6" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D6" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -509,8 +530,11 @@
       <c r="C7" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D7" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -520,8 +544,11 @@
       <c r="C8" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D8" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -531,8 +558,11 @@
       <c r="C9" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D9" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -542,8 +572,11 @@
       <c r="C10" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D10" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -553,8 +586,11 @@
       <c r="C11" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D11" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -564,8 +600,11 @@
       <c r="C12" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D12" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -575,8 +614,11 @@
       <c r="C13" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D13" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>0</v>
       </c>
@@ -586,8 +628,11 @@
       <c r="C14" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D14" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -597,8 +642,11 @@
       <c r="C15" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D15" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>1</v>
       </c>
@@ -608,16 +656,22 @@
       <c r="C16" s="1" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="D16" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>15</v>
       </c>
       <c r="B17" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C17" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D17" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
1 2 4 prez update cviceni navic
</commit_message>
<xml_diff>
--- a/domaciUkoly/odevzdání.xlsx
+++ b/domaciUkoly/odevzdání.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucie Hošková\Desktop\introR_CUNI\domaciUkoly\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B9D549D-D7D4-43A6-9E08-0776603196B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47772242-EEB8-4819-966B-293F7DBFEA8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-83" yWindow="-83" windowWidth="28965" windowHeight="15646" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="odevzdáno" sheetId="1" r:id="rId1"/>
@@ -475,7 +475,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>